<commit_message>
Revised files BPaFF, BFPaT, and PTCF
</commit_message>
<xml_diff>
--- a/InputData/elec/BPaFF/Boolean Peaking and Flexibility Flags.xlsx
+++ b/InputData/elec/BPaFF/Boolean Peaking and Flexibility Flags.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shigu\Documents\_swj\_Talanoa\CPSA Fletcher\dados\InputData (BR) 2024\d08 elec\BPaFF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\elec\BPaFF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01EE8D77-A7E5-4EA6-988C-35AE53A42405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="2436" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4245" yWindow="2430" windowWidth="17280" windowHeight="9960" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="BPaFF-BITPTaP" sheetId="2" r:id="rId2"/>
     <sheet name="BPaFF-BDTPTPF" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -178,7 +177,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -240,9 +239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -280,9 +279,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -317,7 +316,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -352,7 +351,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -525,21 +524,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,7 +546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>42</v>
       </c>
@@ -555,117 +554,117 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -677,30 +676,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
       <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -708,7 +707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -716,15 +715,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -732,7 +731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -740,7 +739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -748,15 +747,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -764,15 +763,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -780,15 +779,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>35</v>
       </c>
       <c r="B13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -796,28 +795,28 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>39</v>
       </c>
       <c r="B15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>40</v>
       </c>
       <c r="B16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -826,30 +825,30 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
       <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -857,7 +856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -865,7 +864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -873,7 +872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -881,7 +880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -889,7 +888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -897,15 +896,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -913,15 +912,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -929,15 +928,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>35</v>
       </c>
       <c r="B13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -945,28 +944,28 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>39</v>
       </c>
       <c r="B15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>40</v>
       </c>
       <c r="B16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>